<commit_message>
continued cleaning the file by adding yellow to students below 2 in their gpa and red if their attendance rate is missing
</commit_message>
<xml_diff>
--- a/Pandas/Datasets/students_clean.xlsx
+++ b/Pandas/Datasets/students_clean.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="students" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,12 +26,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+        <bgColor rgb="00FF0000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +58,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -545,59 +559,59 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>STU01110</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Jeffrey</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  Davis</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>Grade 1</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>jeffrey.davis931@yahoo.com</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>+260-96-9072838</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>2020/09/18</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="1" t="n">
         <v>1.52</v>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
+      <c r="K3" s="1" t="inlineStr"/>
+      <c r="L3" s="1" t="inlineStr">
         <is>
           <t>Morgan Davis</t>
         </is>
       </c>
-      <c r="M3" t="n">
+      <c r="M3" s="1" t="n">
         <v>63.5</v>
       </c>
     </row>
@@ -842,63 +856,63 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>STU02843</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>Christopher</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Brown</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>Grade 1</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="1" t="inlineStr">
         <is>
           <t>christopher_brown@gmail.com</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H8" s="1" t="inlineStr">
         <is>
           <t>0962209692</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" s="1" t="inlineStr">
         <is>
           <t>27 Mar 2023</t>
         </is>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" s="1" t="n">
         <v>1.3</v>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K8" s="1" t="inlineStr">
         <is>
           <t>CHIPATA</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L8" s="1" t="inlineStr">
         <is>
           <t>Vanessa Brown</t>
         </is>
       </c>
-      <c r="M8" t="n">
+      <c r="M8" s="1" t="n">
         <v>70.3</v>
       </c>
     </row>
@@ -1017,59 +1031,59 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>STU01078</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>Tyrone</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>Dennis</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>Grade 1</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="1" t="inlineStr">
         <is>
           <t>tyrone.dennis470@outlook.com</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="1" t="inlineStr">
         <is>
           <t>0979016612</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I11" s="1" t="inlineStr">
         <is>
           <t>2021-03-19</t>
         </is>
       </c>
-      <c r="J11" t="n">
+      <c r="J11" s="1" t="n">
         <v>1.42</v>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K11" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Chingola   </t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="n">
+      <c r="L11" s="1" t="inlineStr"/>
+      <c r="M11" s="1" t="n">
         <v>95.40000000000001</v>
       </c>
     </row>
@@ -1135,63 +1149,63 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>STU03356</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Christopher</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Webb</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Grade 1</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>christopher.webb735@outlook.com</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>0975718099</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>27/01/2020</t>
         </is>
       </c>
-      <c r="J13" t="n">
+      <c r="J13" s="2" t="n">
         <v>3.25</v>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>chingola</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Alexis Webb</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1377,124 +1391,124 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>STU02367</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>William</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>Zuniga</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>Grade 2</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="1" t="inlineStr">
         <is>
           <t>williamz39@gmail.com</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="1" t="inlineStr">
         <is>
           <t>(96) 9367470</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="1" t="inlineStr">
         <is>
           <t>2023/01/15</t>
         </is>
       </c>
-      <c r="J17" t="n">
+      <c r="J17" s="1" t="n">
         <v>1.53</v>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K17" s="1" t="inlineStr">
         <is>
           <t>Ndola</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L17" s="1" t="inlineStr">
         <is>
           <t>Ann Zuniga</t>
         </is>
       </c>
-      <c r="M17" t="n">
+      <c r="M17" s="1" t="n">
         <v>68.5</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>STU04009</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>Kathleen</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>Cole</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>Grade 2</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="1" t="inlineStr">
         <is>
           <t>kathleen.cole957@outlook.com</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H18" s="1" t="inlineStr">
         <is>
           <t>0957848571</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I18" s="1" t="inlineStr">
         <is>
           <t>2023/08/23</t>
         </is>
       </c>
-      <c r="J18" t="n">
+      <c r="J18" s="1" t="n">
         <v>1.69</v>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K18" s="1" t="inlineStr">
         <is>
           <t>Chingola</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L18" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  Isaac Cole</t>
         </is>
       </c>
-      <c r="M18" t="n">
+      <c r="M18" s="1" t="n">
         <v>84.7</v>
       </c>
     </row>
@@ -1556,63 +1570,63 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>STU02049</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Dominique</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>Bailey</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E20" t="n">
+      <c r="E20" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>Grade 2</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="1" t="inlineStr">
         <is>
           <t>dominique.bailey325@outlook.com</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H20" s="1" t="inlineStr">
         <is>
           <t>260950050331</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I20" s="1" t="inlineStr">
         <is>
           <t>2020/04/13</t>
         </is>
       </c>
-      <c r="J20" t="n">
+      <c r="J20" s="1" t="n">
         <v>1.83</v>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K20" s="1" t="inlineStr">
         <is>
           <t>LUSAKA</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L20" s="1" t="inlineStr">
         <is>
           <t>Kristen Bailey</t>
         </is>
       </c>
-      <c r="M20" t="n">
+      <c r="M20" s="1" t="n">
         <v>94.59999999999999</v>
       </c>
     </row>
@@ -1918,122 +1932,122 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>STU03756</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Matthew</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Brooks</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E26" t="n">
+      <c r="E26" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Grade 3</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>matthew_brooks@gmail.com</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>0957121403</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>05/06/2020</t>
         </is>
       </c>
-      <c r="J26" t="n">
+      <c r="J26" s="2" t="n">
         <v>2.2</v>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>Mansa</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>Joseph Brooks</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>STU03638</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Julie</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>Taylor</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E27" t="n">
+      <c r="E27" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>Grade 3</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="1" t="inlineStr">
         <is>
           <t>julie.taylor60@yahoo.com</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" s="1" t="inlineStr">
         <is>
           <t>(97) 4563439</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I27" s="1" t="inlineStr">
         <is>
           <t>17/08/2021</t>
         </is>
       </c>
-      <c r="J27" t="n">
+      <c r="J27" s="1" t="n">
         <v>1.77</v>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K27" s="1" t="inlineStr">
         <is>
           <t>Lusaka</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="L27" s="1" t="inlineStr">
         <is>
           <t>Laura  Taylor</t>
         </is>
       </c>
-      <c r="M27" t="n">
+      <c r="M27" s="1" t="n">
         <v>81.8</v>
       </c>
     </row>
@@ -2697,59 +2711,59 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="1" t="inlineStr">
         <is>
           <t>STU03854</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="1" t="inlineStr">
         <is>
           <t>Amanda</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="1" t="inlineStr">
         <is>
           <t>Rivera</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="1" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E39" t="n">
+      <c r="E39" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="1" t="inlineStr">
         <is>
           <t>Grade 6</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr">
+      <c r="G39" s="1" t="inlineStr"/>
+      <c r="H39" s="1" t="inlineStr">
         <is>
           <t>(97) 5552152</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I39" s="1" t="inlineStr">
         <is>
           <t>2021/12/20</t>
         </is>
       </c>
-      <c r="J39" t="n">
+      <c r="J39" s="1" t="n">
         <v>1.34</v>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="K39" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  Lusaka</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="L39" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  Justin Rivera</t>
         </is>
       </c>
-      <c r="M39" t="n">
+      <c r="M39" s="1" t="n">
         <v>80.59999999999999</v>
       </c>
     </row>
@@ -2815,59 +2829,59 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="1" t="inlineStr">
         <is>
           <t>STU02007</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Joshua   </t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="1" t="inlineStr">
         <is>
           <t>Smith</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="1" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="E41" t="n">
+      <c r="E41" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="1" t="inlineStr">
         <is>
           <t>Grade 6</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr">
+      <c r="G41" s="1" t="inlineStr"/>
+      <c r="H41" s="1" t="inlineStr">
         <is>
           <t>0954277885</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I41" s="1" t="inlineStr">
         <is>
           <t>2018/09/24</t>
         </is>
       </c>
-      <c r="J41" t="n">
+      <c r="J41" s="1" t="n">
         <v>1.32</v>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K41" s="1" t="inlineStr">
         <is>
           <t>Solwezi</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="L41" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Kimberly Smith   </t>
         </is>
       </c>
-      <c r="M41" t="n">
+      <c r="M41" s="1" t="n">
         <v>89.7</v>
       </c>
     </row>
@@ -2933,63 +2947,63 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="1" t="inlineStr">
         <is>
           <t>STU03844</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="1" t="inlineStr">
         <is>
           <t>Eric</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  Richardson</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="1" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E43" t="n">
+      <c r="E43" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="1" t="inlineStr">
         <is>
           <t>Grade 6</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G43" s="1" t="inlineStr">
         <is>
           <t>eric.richardson577@outlook.com</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H43" s="1" t="inlineStr">
         <is>
           <t>+260-95-8992886</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I43" s="1" t="inlineStr">
         <is>
           <t>08-16-2021</t>
         </is>
       </c>
-      <c r="J43" t="n">
+      <c r="J43" s="1" t="n">
         <v>1.65</v>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K43" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Ndola   </t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="L43" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  Jordan Richardson</t>
         </is>
       </c>
-      <c r="M43" t="n">
+      <c r="M43" s="1" t="n">
         <v>77.90000000000001</v>
       </c>
     </row>
@@ -3055,63 +3069,63 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="1" t="inlineStr">
         <is>
           <t>STU00277</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="1" t="inlineStr">
         <is>
           <t>Megan</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="1" t="inlineStr">
         <is>
           <t>Adams</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="1" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E45" t="n">
+      <c r="E45" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="1" t="inlineStr">
         <is>
           <t>Grade 6</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G45" s="1" t="inlineStr">
         <is>
           <t>megan.adams182@school.edu.zm</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H45" s="1" t="inlineStr">
         <is>
           <t>260960168488</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I45" s="1" t="inlineStr">
         <is>
           <t>04 Nov 2019</t>
         </is>
       </c>
-      <c r="J45" t="n">
+      <c r="J45" s="1" t="n">
         <v>1.94</v>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K45" s="1" t="inlineStr">
         <is>
           <t>Solwezi</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="L45" s="1" t="inlineStr">
         <is>
           <t>Kelly Adams</t>
         </is>
       </c>
-      <c r="M45" t="n">
+      <c r="M45" s="1" t="n">
         <v>82.2</v>
       </c>
     </row>
@@ -3238,120 +3252,120 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="1" t="inlineStr">
         <is>
           <t>STU02155</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="1" t="inlineStr">
         <is>
           <t>Glenn</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="1" t="inlineStr">
         <is>
           <t>Wright</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="1" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E48" t="n">
+      <c r="E48" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="1" t="inlineStr">
         <is>
           <t>Grade 7</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr">
+      <c r="G48" s="1" t="inlineStr"/>
+      <c r="H48" s="1" t="inlineStr">
         <is>
           <t>+260-95-2313269</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="I48" s="1" t="inlineStr">
         <is>
           <t>18/11/2019</t>
         </is>
       </c>
-      <c r="J48" t="n">
+      <c r="J48" s="1" t="n">
         <v>1.74</v>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="K48" s="1" t="inlineStr">
         <is>
           <t>Chipata</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr">
+      <c r="L48" s="1" t="inlineStr">
         <is>
           <t>John Wright</t>
         </is>
       </c>
-      <c r="M48" t="n">
+      <c r="M48" s="1" t="n">
         <v>91.40000000000001</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="1" t="inlineStr">
         <is>
           <t>STU00389</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="1" t="inlineStr">
         <is>
           <t>Eric</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="1" t="inlineStr">
         <is>
           <t>Parker</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="1" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E49" t="n">
+      <c r="E49" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F49" s="1" t="inlineStr">
         <is>
           <t>Grade 7</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="G49" s="1" t="inlineStr">
         <is>
           <t>eric.parker190@school.edu.zm</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="H49" s="1" t="inlineStr">
         <is>
           <t>+260-97-9229532</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="I49" s="1" t="inlineStr">
         <is>
           <t>01-09-2020</t>
         </is>
       </c>
-      <c r="J49" t="n">
+      <c r="J49" s="1" t="n">
         <v>1.49</v>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="K49" s="1" t="inlineStr">
         <is>
           <t>Kitwe</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="L49" s="1" t="inlineStr">
         <is>
           <t>Mark Parker</t>
         </is>
       </c>
-      <c r="M49" t="n">
+      <c r="M49" s="1" t="n">
         <v>77.09999999999999</v>
       </c>
     </row>
@@ -3474,124 +3488,124 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="1" t="inlineStr">
         <is>
           <t>STU00854</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Nicholas   </t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="1" t="inlineStr">
         <is>
           <t>Matthews</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="1" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="E52" t="n">
+      <c r="E52" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F52" s="1" t="inlineStr">
         <is>
           <t>Grade 7</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="G52" s="1" t="inlineStr">
         <is>
           <t>nicholas.matthews24@yahoo.com</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="H52" s="1" t="inlineStr">
         <is>
           <t>+260-97-6924408</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="I52" s="1" t="inlineStr">
         <is>
           <t>2021-07-17</t>
         </is>
       </c>
-      <c r="J52" t="n">
+      <c r="J52" s="1" t="n">
         <v>1.39</v>
       </c>
-      <c r="K52" t="inlineStr">
+      <c r="K52" s="1" t="inlineStr">
         <is>
           <t>solwezi</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr">
+      <c r="L52" s="1" t="inlineStr">
         <is>
           <t>Jason Matthews</t>
         </is>
       </c>
-      <c r="M52" t="n">
+      <c r="M52" s="1" t="n">
         <v>82.3</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="1" t="inlineStr">
         <is>
           <t>STU03665</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="1" t="inlineStr">
         <is>
           <t>Maria</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="1" t="inlineStr">
         <is>
           <t>Ramos</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="1" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E53" t="n">
+      <c r="E53" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F53" s="1" t="inlineStr">
         <is>
           <t>Grade 7</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G53" s="1" t="inlineStr">
         <is>
           <t>maria_ramos@school.edu.zm</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="H53" s="1" t="inlineStr">
         <is>
           <t>0953022756</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="I53" s="1" t="inlineStr">
         <is>
           <t>11-12-2022</t>
         </is>
       </c>
-      <c r="J53" t="n">
+      <c r="J53" s="1" t="n">
         <v>1.38</v>
       </c>
-      <c r="K53" t="inlineStr">
+      <c r="K53" s="1" t="inlineStr">
         <is>
           <t>CHINGOLA</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr">
+      <c r="L53" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Kimberly Ramos   </t>
         </is>
       </c>
-      <c r="M53" t="n">
+      <c r="M53" s="1" t="n">
         <v>75.2</v>
       </c>
     </row>
@@ -3657,63 +3671,63 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="1" t="inlineStr">
         <is>
           <t>STU04241</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Grace   </t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Valentine   </t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="1" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E55" t="n">
+      <c r="E55" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F55" s="1" t="inlineStr">
         <is>
           <t>Grade 8</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
+      <c r="G55" s="1" t="inlineStr">
         <is>
           <t>grace_valentine@gmail.com</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
+      <c r="H55" s="1" t="inlineStr">
         <is>
           <t>(95) 1764359</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
+      <c r="I55" s="1" t="inlineStr">
         <is>
           <t>2019/01/12</t>
         </is>
       </c>
-      <c r="J55" t="n">
+      <c r="J55" s="1" t="n">
         <v>1.27</v>
       </c>
-      <c r="K55" t="inlineStr">
+      <c r="K55" s="1" t="inlineStr">
         <is>
           <t>mansa</t>
         </is>
       </c>
-      <c r="L55" t="inlineStr">
+      <c r="L55" s="1" t="inlineStr">
         <is>
           <t>Michael  Valentine</t>
         </is>
       </c>
-      <c r="M55" t="n">
+      <c r="M55" s="1" t="n">
         <v>75.90000000000001</v>
       </c>
     </row>
@@ -3779,63 +3793,63 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="1" t="inlineStr">
         <is>
           <t>STU01942</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="1" t="inlineStr">
         <is>
           <t>Kathy</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="1" t="inlineStr">
         <is>
           <t>Chambers</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="1" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="E57" t="n">
+      <c r="E57" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F57" s="1" t="inlineStr">
         <is>
           <t>Grade 8</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="G57" s="1" t="inlineStr">
         <is>
           <t>kathyc2@yahoo.com</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="H57" s="1" t="inlineStr">
         <is>
           <t>0957699314</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
+      <c r="I57" s="1" t="inlineStr">
         <is>
           <t>07/05/2021</t>
         </is>
       </c>
-      <c r="J57" t="n">
+      <c r="J57" s="1" t="n">
         <v>1.15</v>
       </c>
-      <c r="K57" t="inlineStr">
+      <c r="K57" s="1" t="inlineStr">
         <is>
           <t>Mansa</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr">
+      <c r="L57" s="1" t="inlineStr">
         <is>
           <t>Jacob Chambers</t>
         </is>
       </c>
-      <c r="M57" t="n">
+      <c r="M57" s="1" t="n">
         <v>79.8</v>
       </c>
     </row>
@@ -4261,124 +4275,124 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="1" t="inlineStr">
         <is>
           <t>STU02955</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Jeffrey   </t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="1" t="inlineStr">
         <is>
           <t>Obrien</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" s="1" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E65" t="n">
+      <c r="E65" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" s="1" t="inlineStr">
         <is>
           <t>Grade 10</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
+      <c r="G65" s="1" t="inlineStr">
         <is>
           <t>jeffrey.obrien701@outlook.com</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="H65" s="1" t="inlineStr">
         <is>
           <t>0974117026</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr">
+      <c r="I65" s="1" t="inlineStr">
         <is>
           <t>06/03/2019</t>
         </is>
       </c>
-      <c r="J65" t="n">
+      <c r="J65" s="1" t="n">
         <v>1.05</v>
       </c>
-      <c r="K65" t="inlineStr">
+      <c r="K65" s="1" t="inlineStr">
         <is>
           <t>Chipata</t>
         </is>
       </c>
-      <c r="L65" t="inlineStr">
+      <c r="L65" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Melissa Obrien   </t>
         </is>
       </c>
-      <c r="M65" t="n">
+      <c r="M65" s="1" t="n">
         <v>96.7</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>STU02596</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  David</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>Jacobson</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="E66" t="n">
+      <c r="E66" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>Grade 10</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr">
         <is>
           <t>david_jacobson@school.edu.zm</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>+260-95-8348268</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr">
+      <c r="I66" s="2" t="inlineStr">
         <is>
           <t>03 Apr 2023</t>
         </is>
       </c>
-      <c r="J66" t="n">
+      <c r="J66" s="2" t="n">
         <v>3.99</v>
       </c>
-      <c r="K66" t="inlineStr">
+      <c r="K66" s="2" t="inlineStr">
         <is>
           <t>MONGU</t>
         </is>
       </c>
-      <c r="L66" t="inlineStr">
+      <c r="L66" s="2" t="inlineStr">
         <is>
           <t>Zachary Jacobson</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr"/>
+      <c r="M66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4499,63 +4513,63 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="1" t="inlineStr">
         <is>
           <t>STU01881</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="1" t="inlineStr">
         <is>
           <t>John</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="1" t="inlineStr">
         <is>
           <t>Short</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D69" s="1" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E69" t="n">
+      <c r="E69" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F69" s="1" t="inlineStr">
         <is>
           <t>Grade 10</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
+      <c r="G69" s="1" t="inlineStr">
         <is>
           <t>jacqueline.thompson387@yahoo.com</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr">
+      <c r="H69" s="1" t="inlineStr">
         <is>
           <t>+260-97-1667503</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
+      <c r="I69" s="1" t="inlineStr">
         <is>
           <t>30 May 2022</t>
         </is>
       </c>
-      <c r="J69" t="n">
+      <c r="J69" s="1" t="n">
         <v>1.92</v>
       </c>
-      <c r="K69" t="inlineStr">
+      <c r="K69" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  Chingola</t>
         </is>
       </c>
-      <c r="L69" t="inlineStr">
+      <c r="L69" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Jeffrey Short   </t>
         </is>
       </c>
-      <c r="M69" t="n">
+      <c r="M69" s="1" t="n">
         <v>78.90000000000001</v>
       </c>
     </row>
@@ -4804,246 +4818,246 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" s="1" t="inlineStr">
         <is>
           <t>STU03341</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B74" s="1" t="inlineStr">
         <is>
           <t>Michelle</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C74" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  Roberts</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D74" s="1" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="E74" t="n">
+      <c r="E74" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="F74" s="1" t="inlineStr">
         <is>
           <t>Grade 11</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr">
+      <c r="G74" s="1" t="inlineStr">
         <is>
           <t>michelle.roberts370@gmail.com</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr">
+      <c r="H74" s="1" t="inlineStr">
         <is>
           <t>+260-95-4739571</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr">
+      <c r="I74" s="1" t="inlineStr">
         <is>
           <t>2018/03/19</t>
         </is>
       </c>
-      <c r="J74" t="n">
+      <c r="J74" s="1" t="n">
         <v>1.46</v>
       </c>
-      <c r="K74" t="inlineStr">
+      <c r="K74" s="1" t="inlineStr">
         <is>
           <t>Chipata</t>
         </is>
       </c>
-      <c r="L74" t="inlineStr">
+      <c r="L74" s="1" t="inlineStr">
         <is>
           <t>Bryan Roberts</t>
         </is>
       </c>
-      <c r="M74" t="n">
+      <c r="M74" s="1" t="n">
         <v>89</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="1" t="inlineStr">
         <is>
           <t>STU00915</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Joseph   </t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="1" t="inlineStr">
         <is>
           <t>Roberts</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D75" s="1" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E75" t="n">
+      <c r="E75" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F75" s="1" t="inlineStr">
         <is>
           <t>Grade 11</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
+      <c r="G75" s="1" t="inlineStr">
         <is>
           <t>joseph.roberts878@gmail.com</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr">
+      <c r="H75" s="1" t="inlineStr">
         <is>
           <t>(95) 7735594</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr">
+      <c r="I75" s="1" t="inlineStr">
         <is>
           <t>2022-12-19</t>
         </is>
       </c>
-      <c r="J75" t="n">
+      <c r="J75" s="1" t="n">
         <v>1.62</v>
       </c>
-      <c r="K75" t="inlineStr">
+      <c r="K75" s="1" t="inlineStr">
         <is>
           <t>ndola</t>
         </is>
       </c>
-      <c r="L75" t="inlineStr">
+      <c r="L75" s="1" t="inlineStr">
         <is>
           <t>Jacob Roberts</t>
         </is>
       </c>
-      <c r="M75" t="n">
+      <c r="M75" s="1" t="n">
         <v>87</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="1" t="inlineStr">
         <is>
           <t>STU04454</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="1" t="inlineStr">
         <is>
           <t>Robin</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C76" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Watson   </t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D76" s="1" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="E76" t="n">
+      <c r="E76" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F76" s="1" t="inlineStr">
         <is>
           <t>Grade 11</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
+      <c r="G76" s="1" t="inlineStr">
         <is>
           <t>robin_watson@gmail.com</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr">
+      <c r="H76" s="1" t="inlineStr">
         <is>
           <t>260962432072</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr">
+      <c r="I76" s="1" t="inlineStr">
         <is>
           <t>2022/04/30</t>
         </is>
       </c>
-      <c r="J76" t="n">
+      <c r="J76" s="1" t="n">
         <v>1.44</v>
       </c>
-      <c r="K76" t="inlineStr">
+      <c r="K76" s="1" t="inlineStr">
         <is>
           <t>Kabwe</t>
         </is>
       </c>
-      <c r="L76" t="inlineStr">
+      <c r="L76" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  Anthony Watson</t>
         </is>
       </c>
-      <c r="M76" t="n">
+      <c r="M76" s="1" t="n">
         <v>91.59999999999999</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="A77" s="1" t="inlineStr">
         <is>
           <t>STU01032</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="1" t="inlineStr">
         <is>
           <t>Loretta</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C77" s="1" t="inlineStr">
         <is>
           <t>Foster</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D77" s="1" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E77" t="n">
+      <c r="E77" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="F77" s="1" t="inlineStr">
         <is>
           <t>Grade 12</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr">
+      <c r="G77" s="1" t="inlineStr">
         <is>
           <t>loretta_foster@gmail.com</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr">
+      <c r="H77" s="1" t="inlineStr">
         <is>
           <t>260974160580</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr">
+      <c r="I77" s="1" t="inlineStr">
         <is>
           <t>10-23-2023</t>
         </is>
       </c>
-      <c r="J77" t="n">
+      <c r="J77" s="1" t="n">
         <v>1.81</v>
       </c>
-      <c r="K77" t="inlineStr">
+      <c r="K77" s="1" t="inlineStr">
         <is>
           <t>Solwezi</t>
         </is>
       </c>
-      <c r="L77" t="inlineStr">
+      <c r="L77" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Juan Foster   </t>
         </is>
       </c>
-      <c r="M77" t="n">
+      <c r="M77" s="1" t="n">
         <v>99.7</v>
       </c>
     </row>
@@ -5530,61 +5544,61 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
+      <c r="A86" s="1" t="inlineStr">
         <is>
           <t>STU01514</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B86" s="1" t="inlineStr">
         <is>
           <t>Henry</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C86" s="1" t="inlineStr">
         <is>
           <t>Lee</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D86" s="1" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
-      <c r="F86" t="inlineStr">
+      <c r="E86" s="1" t="inlineStr"/>
+      <c r="F86" s="1" t="inlineStr">
         <is>
           <t>Grade 7</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr">
+      <c r="G86" s="1" t="inlineStr">
         <is>
           <t>henry_lee@gmail.com</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
+      <c r="H86" s="1" t="inlineStr">
         <is>
           <t>0978851786</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr">
+      <c r="I86" s="1" t="inlineStr">
         <is>
           <t>2022-05-28</t>
         </is>
       </c>
-      <c r="J86" t="n">
+      <c r="J86" s="1" t="n">
         <v>1.98</v>
       </c>
-      <c r="K86" t="inlineStr">
+      <c r="K86" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  LUSAKA</t>
         </is>
       </c>
-      <c r="L86" t="inlineStr">
+      <c r="L86" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">  Denise Lee</t>
         </is>
       </c>
-      <c r="M86" t="n">
+      <c r="M86" s="1" t="n">
         <v>75.59999999999999</v>
       </c>
     </row>

</xml_diff>